<commit_message>
Update berita 2026-08-03 09:04 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-01.xlsx
+++ b/data/berita_antara_2026-08-01.xlsx
@@ -504,66 +504,66 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ekonomi, otomotif</t>
+          <t>photo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jam buka GIIAS 2026 lengkap, simak jadwal operasional dan harga tiket</t>
+          <t>Begini kemeriahan Jakarta Watersport Festival 2026 di Danau Sunter</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 14:57:18 +0700</t>
+          <t>Sat, 01 Aug 2026 18:01:11 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Pameran otomotif Gaikindo Indonesia International Auto Show (GIIAS) 2026 resmi digelar pada 30 Juli hingga 9 Agustus ...</t>
+          <t>Peserta beradu kecepatan saat mengikuti lomba perahu naga pada Jakarta Watersport Festival 2026 di Danau Sunter, Jakarta.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5675691/jam-buka-giias-2026-lengkap-simak-jadwal-operasional-dan-harga-tiket</t>
+          <t>https://www.antaranews.com/foto/5675857/begini-kemeriahan-jakarta-watersport-festival-2026-di-danau-sunter</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/IMG_1452.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Jakarta-Watersport-Festival-2026-182026-pma-2.jpg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>ekonomi, otomotif</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LPDB siapkan KDKMP di Papua agar layak memperoleh pembiayaan</t>
+          <t>Jam buka GIIAS 2026 lengkap, simak jadwal operasional dan harga tiket</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 16:45:47 +0700</t>
+          <t>Sat, 01 Aug 2026 14:57:18 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lembaga Pengelola Dana Bergulir (LPDB) Koperasi memperkuat kapasitas 15 Koperasi Desa/Kelurahan Merah Putih (KDKMP) ...</t>
+          <t>Pameran otomotif Gaikindo Indonesia International Auto Show (GIIAS) 2026 resmi digelar pada 30 Juli hingga 9 Agustus ...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675779/lpdb-siapkan-kdkmp-di-papua-agar-layak-memperoleh-pembiayaan</t>
+          <t>https://otomotif.antaranews.com/berita/5675691/jam-buka-giias-2026-lengkap-simak-jadwal-operasional-dan-harga-tiket</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/WhatsApp-Image-2026-08-01-at-16.36.12.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/IMG_1452.jpg</t>
         </is>
       </c>
     </row>
@@ -575,28 +575,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Apkasi usulkan formula DBH berbasis produksi perkuat fiskal daerah</t>
+          <t>LPDB siapkan KDKMP di Papua agar layak memperoleh pembiayaan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 14:59:10 +0700</t>
+          <t>Sat, 01 Aug 2026 16:45:47 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Asosiasi Pemerintah Kabupaten Seluruh Indonesia (Apkasi) mengusulkan penyempurnaan formula Dana Bagi Hasil (DBH) sektor ...</t>
+          <t>Lembaga Pengelola Dana Bergulir (LPDB) Koperasi memperkuat kapasitas 15 Koperasi Desa/Kelurahan Merah Putih (KDKMP) ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675695/apkasi-usulkan-formula-dbh-berbasis-produksi-perkuat-fiskal-daerah</t>
+          <t>https://www.antaranews.com/berita/5675779/lpdb-siapkan-kdkmp-di-papua-agar-layak-memperoleh-pembiayaan</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/1000175928.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/WhatsApp-Image-2026-08-01-at-16.36.12.jpeg</t>
         </is>
       </c>
     </row>
@@ -608,28 +608,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gubernur Khofifah beri keringanan pajak kendaraan selama Agustus 2026</t>
+          <t>Apkasi usulkan formula DBH berbasis produksi perkuat fiskal daerah</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 10:03:39 +0700</t>
+          <t>Sat, 01 Aug 2026 14:59:10 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Gubernur Jawa Timur Khofifah Indar Parawansa memberikan keringanan pembayaran pajak kendaraan selama periode 1-31 ...</t>
+          <t>Asosiasi Pemerintah Kabupaten Seluruh Indonesia (Apkasi) mengusulkan penyempurnaan formula Dana Bagi Hasil (DBH) sektor ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675479/gubernur-khofifah-beri-keringanan-pajak-kendaraan-selama-agustus-2026</t>
+          <t>https://www.antaranews.com/berita/5675695/apkasi-usulkan-formula-dbh-berbasis-produksi-perkuat-fiskal-daerah</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/1311386.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/1000175928.jpg</t>
         </is>
       </c>
     </row>
@@ -641,61 +641,61 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Maybank Indonesia bukukan laba bersih Rp698 miliar semester I-2026</t>
+          <t>Gubernur Khofifah beri keringanan pajak kendaraan selama Agustus 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 00:09:43 +0700</t>
+          <t>Sat, 01 Aug 2026 10:03:39 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PT Bank Maybank Indonesia Tbk (Maybank Indonesia) membukukan laba bersih sebesar Rp698 miliar pada semester I-2026, ...</t>
+          <t>Gubernur Jawa Timur Khofifah Indar Parawansa memberikan keringanan pembayaran pajak kendaraan selama periode 1-31 ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675279/maybank-indonesia-bukukan-laba-bersih-rp698-miliar-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5675479/gubernur-khofifah-beri-keringanan-pajak-kendaraan-selama-agustus-2026</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/05/02/Sentra-Senayan-Picture-Night-Time-1_2.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/1311386.jpg</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pemerintah RI targetkan stop impor garam per akhir 2027</t>
+          <t>Maybank Indonesia bukukan laba bersih Rp698 miliar semester I-2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 07:13:28 +0700</t>
+          <t>Sat, 01 Aug 2026 00:09:43 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Pemerintah Republik Indonesia (RI) menargetkan untuk menyetop impor garam per akhir 2027 sebagai bagian dari upaya ...</t>
+          <t>PT Bank Maybank Indonesia Tbk (Maybank Indonesia) membukukan laba bersih sebesar Rp698 miliar pada semester I-2026, ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675401/pemerintah-ri-targetkan-stop-impor-garam-per-akhir-2027</t>
+          <t>https://www.antaranews.com/berita/5675279/maybank-indonesia-bukukan-laba-bersih-rp698-miliar-semester-i-2026</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/CjkinzN000023_20260731_CBMFN0A001.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/05/02/Sentra-Senayan-Picture-Night-Time-1_2.jpg</t>
         </is>
       </c>
     </row>
@@ -707,94 +707,94 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IMIP raih penghargaan utama ESG IDX Channel 2026</t>
+          <t>Pemerintah RI targetkan stop impor garam per akhir 2027</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 07:10:53 +0700</t>
+          <t>Sat, 01 Aug 2026 07:13:28 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Kawasan Industri Indonesia Morowali Industrial Park (IMIP) berhasil meraih Penghargaan Utama ESG untuk sektor ...</t>
+          <t>Pemerintah Republik Indonesia (RI) menargetkan untuk menyetop impor garam per akhir 2027 sebagai bagian dari upaya ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675396/imip-raih-penghargaan-utama-esg-idx-channel-2026</t>
+          <t>https://www.antaranews.com/berita/5675401/pemerintah-ri-targetkan-stop-impor-garam-per-akhir-2027</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/CjkinzN000028_20260731_CBMFN0A001.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/CjkinzN000023_20260731_CBMFN0A001.jpg</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>humaniora</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hukum mengedarkan kotak amal saat khutbah Jumat, makruh atau boleh?</t>
+          <t>IMIP raih penghargaan utama ESG IDX Channel 2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 14:48:54 +0700</t>
+          <t>Sat, 01 Aug 2026 07:10:53 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Mengedarkan kotak amal ketika khutbah Jumat berlangsung menjadi kebiasaan yang masih ditemukan di sejumlah masjid. ...</t>
+          <t>Kawasan Industri Indonesia Morowali Industrial Park (IMIP) berhasil meraih Penghargaan Utama ESG untuk sektor ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675680/hukum-mengedarkan-kotak-amal-saat-khutbah-jumat-makruh-atau-boleh</t>
+          <t>https://www.antaranews.com/berita/5675396/imip-raih-penghargaan-utama-esg-idx-channel-2026</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/02/20/shalat-jumat-pertama-ramadhan-di-masjid-kuno-indrapuri-aceh-2734630.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/CjkinzN000028_20260731_CBMFN0A001.jpg</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>lifestyle</t>
+          <t>humaniora</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>6 wisata alam di Bogor yang ramah lansia, nyaman dan mudah diakses</t>
+          <t>Hukum mengedarkan kotak amal saat khutbah Jumat, makruh atau boleh?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 15:08:07 +0700</t>
+          <t>Sat, 01 Aug 2026 14:48:54 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Kota Bogor dan wilayah sekitarnya menawarkan sejumlah destinasi wisata alam yang cocok dikunjungi bersama lansia. ...</t>
+          <t>Mengedarkan kotak amal ketika khutbah Jumat berlangsung menjadi kebiasaan yang masih ditemukan di sejumlah masjid. ...</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675711/6-wisata-alam-di-bogor-yang-ramah-lansia-nyaman-dan-mudah-diakses</t>
+          <t>https://www.antaranews.com/berita/5675680/hukum-mengedarkan-kotak-amal-saat-khutbah-jumat-makruh-atau-boleh</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/18/hut-krb-6.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/20/shalat-jumat-pertama-ramadhan-di-masjid-kuno-indrapuri-aceh-2734630.jpg</t>
         </is>
       </c>
     </row>
@@ -806,28 +806,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cara menghilangkan rasa panas di tangan akibat cabai</t>
+          <t>6 wisata alam di Bogor yang ramah lansia, nyaman dan mudah diakses</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 15:02:01 +0700</t>
+          <t>Sat, 01 Aug 2026 15:08:07 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sensasi panas pada tangan setelah memegang atau mengolah cabai sering membuat tidak nyaman. Kondisi tersebut terjadi ...</t>
+          <t>Kota Bogor dan wilayah sekitarnya menawarkan sejumlah destinasi wisata alam yang cocok dikunjungi bersama lansia. ...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675701/cara-menghilangkan-rasa-panas-di-tangan-akibat-cabai</t>
+          <t>https://www.antaranews.com/berita/5675711/6-wisata-alam-di-bogor-yang-ramah-lansia-nyaman-dan-mudah-diakses</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/10/04/cuci-tangan.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/18/hut-krb-6.jpg</t>
         </is>
       </c>
     </row>
@@ -839,61 +839,61 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10 kebiasaan kecil yang bisa meningkatkan kualitas hidup sehari-hari</t>
+          <t>Cara menghilangkan rasa panas di tangan akibat cabai</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 14:53:11 +0700</t>
+          <t>Sat, 01 Aug 2026 15:02:01 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Menjalani hidup yang lebih baik tidak selalu membutuhkan perubahan besar. Justru, kebiasaan-kebiasaan kecil yang ...</t>
+          <t>Sensasi panas pada tangan setelah memegang atau mengolah cabai sering membuat tidak nyaman. Kondisi tersebut terjadi ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5675683/10-kebiasaan-kecil-yang-bisa-meningkatkan-kualitas-hidup-sehari-hari</t>
+          <t>https://www.antaranews.com/berita/5675701/cara-menghilangkan-rasa-panas-di-tangan-akibat-cabai</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/24/skrining-kebugaran-jasmani-asn-kota-bogor-2810969.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/10/04/cuci-tangan.jpg</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>photo</t>
+          <t>lifestyle</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kalahkan Port FC 2-1, Persebaya melaju ke semifinal Piala Presiden 2026</t>
+          <t>10 kebiasaan kecil yang bisa meningkatkan kualitas hidup sehari-hari</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 22:35:05 +0700</t>
+          <t>Sat, 01 Aug 2026 14:53:11 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pesepak bola Persebaya Surabaya Miguel Pereira (bawah) bersama rekannya Koko Ari Araya (atas) berselebrasi usai mencetak gol ke gawang Port FC pada pertandingan Grup B Piala Presiden 2026 di Stadion Gelora Bung Tomo, Surabaya, Jawa Timur, Sabtu (1/8/2026). Persebaya Surabaya lolos ke semifinal usai mengalahkan Port FC dengan skor 2-1. ANTARA FOTO/Rizal Hanafi/YU</t>
+          <t>Menjalani hidup yang lebih baik tidak selalu membutuhkan perubahan besar. Justru, kebiasaan-kebiasaan kecil yang ...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676144/kalahkan-port-fc-2-1-persebaya-melaju-ke-semifinal-piala-presiden-2026</t>
+          <t>https://www.antaranews.com/berita/5675683/10-kebiasaan-kecil-yang-bisa-meningkatkan-kualitas-hidup-sehari-hari</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Persebaya-Menang-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/24/skrining-kebugaran-jasmani-asn-kota-bogor-2810969.jpg</t>
         </is>
       </c>
     </row>
@@ -905,28 +905,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Zikir dan doa kebangsaan sambut HUT ke-81 RI</t>
+          <t>Kalahkan Port FC 2-1, Persebaya melaju ke semifinal Piala Presiden 2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 22:00:30 +0700</t>
+          <t>Sat, 01 Aug 2026 22:35:05 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Umat Islam mengikuti zikir dan doa kebangsaan 2006 di kawasan Monas, Jakarta.</t>
+          <t>Pesepak bola Persebaya Surabaya Miguel Pereira (bawah) bersama rekannya Koko Ari Araya (atas) berselebrasi usai mencetak gol ke gawang Port FC pada pertandingan Grup B Piala Presiden 2026 di Stadion Gelora Bung Tomo, Surabaya, Jawa Timur, Sabtu (1/8/2026). Persebaya Surabaya lolos ke semifinal usai mengalahkan Port FC dengan skor 2-1. ANTARA FOTO/Rizal Hanafi/YU</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676104/zikir-dan-doa-kebangsaan-sambut-hut-ke-81-ri</t>
+          <t>https://www.antaranews.com/foto/5676144/kalahkan-port-fc-2-1-persebaya-melaju-ke-semifinal-piala-presiden-2026</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Zikir-3.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Persebaya-Menang-1.jpg</t>
         </is>
       </c>
     </row>
@@ -938,28 +938,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Aston Villa kalahkan Indonesia All Stars dengan skor 3-1</t>
+          <t>Zikir dan doa kebangsaan sambut HUT ke-81 RI</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 21:43:10 +0700</t>
+          <t>Sat, 01 Aug 2026 22:00:30 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pesepak bola Indonesia All Stars Oliver Leeming (kanan) melakukan duel udara dengan pesepak bola Aston Villa Triston Rowe (kedua kanan) pada pertandingan bertajuk Aston Villa Pre-Season Tour Indonesia 2026 di Stadion Utama Gelora Bung Karno, Senayan, Jakarta, Sabtu (1/8/2026). Indonesia All Stars dikalahkan Aston Villa dengan skor 1-3 ANTARA FOTO/Fauzan/YU</t>
+          <t>Umat Islam mengikuti zikir dan doa kebangsaan 2006 di kawasan Monas, Jakarta.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676091/aston-villa-kalahkan-indonesia-all-stars-dengan-skor-3-1</t>
+          <t>https://www.antaranews.com/foto/5676104/zikir-dan-doa-kebangsaan-sambut-hut-ke-81-ri</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Indoesia-All-Star-vs-Aston-Vila-2.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Zikir-3.jpg</t>
         </is>
       </c>
     </row>
@@ -971,28 +971,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Begini kondisi kebakaran lahan di Indralaya Utara Sumsel</t>
+          <t>Aston Villa kalahkan Indonesia All Stars dengan skor 3-1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 21:32:25 +0700</t>
+          <t>Sat, 01 Aug 2026 21:43:10 +0700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Foto udara petugas bersama warga berusaha memadamkan kebakaran lahan yang berada di dekat rumahnya di Desa Sungai Rambutan, Indralaya Utara, Ogan Ili (OI), Sumatera Selatan.</t>
+          <t>Pesepak bola Indonesia All Stars Oliver Leeming (kanan) melakukan duel udara dengan pesepak bola Aston Villa Triston Rowe (kedua kanan) pada pertandingan bertajuk Aston Villa Pre-Season Tour Indonesia 2026 di Stadion Utama Gelora Bung Karno, Senayan, Jakarta, Sabtu (1/8/2026). Indonesia All Stars dikalahkan Aston Villa dengan skor 1-3 ANTARA FOTO/Fauzan/YU</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676076/begini-kondisi-kebakaran-lahan-di-indralaya-utara-sumsel</t>
+          <t>https://www.antaranews.com/foto/5676091/aston-villa-kalahkan-indonesia-all-stars-dengan-skor-3-1</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Kebakaran-Lahan-4.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Indoesia-All-Star-vs-Aston-Vila-2.jpg</t>
         </is>
       </c>
     </row>
@@ -1004,28 +1004,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sudah sepekan petugas berjibaku padamkan karhutla di Kubu Raya</t>
+          <t>Begini kondisi kebakaran lahan di Indralaya Utara Sumsel</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 20:51:18 +0700</t>
+          <t>Sat, 01 Aug 2026 21:32:25 +0700</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Personel BPBD Kabupaten Kubu Raya menyemprotkan air ke lahan gambut yang terbakar di Dusun Sidomulyo, Desa Limbung, Kecamatan Sungai Raya, Kabupaten Kubu Raya, Kalimantan Barat.</t>
+          <t>Foto udara petugas bersama warga berusaha memadamkan kebakaran lahan yang berada di dekat rumahnya di Desa Sungai Rambutan, Indralaya Utara, Ogan Ili (OI), Sumatera Selatan.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676039/sudah-sepekan-petugas-berjibaku-padamkan-karhutla-di-kubu-raya</t>
+          <t>https://www.antaranews.com/foto/5676076/begini-kondisi-kebakaran-lahan-di-indralaya-utara-sumsel</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Kebakaran-2.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Kebakaran-Lahan-4.jpg</t>
         </is>
       </c>
     </row>
@@ -1037,28 +1037,28 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Pergelaran kesenian balaganjur pada hari suci umat Hindu di Bali</t>
+          <t>Sudah sepekan petugas berjibaku padamkan karhutla di Kubu Raya</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 20:11:17 +0700</t>
+          <t>Sat, 01 Aug 2026 20:51:18 +0700</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sejumlah pemuda menampilkan kesenian baleganjur pada Hari Suci Tumpek Krulut di The Blooms Bali, Tabanan, Bali.</t>
+          <t>Personel BPBD Kabupaten Kubu Raya menyemprotkan air ke lahan gambut yang terbakar di Dusun Sidomulyo, Desa Limbung, Kecamatan Sungai Raya, Kabupaten Kubu Raya, Kalimantan Barat.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5676007/pergelaran-kesenian-balaganjur-pada-hari-suci-umat-hindu-di-bali</t>
+          <t>https://www.antaranews.com/foto/5676039/sudah-sepekan-petugas-berjibaku-padamkan-karhutla-di-kubu-raya</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Bali-2.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Kebakaran-2.jpg</t>
         </is>
       </c>
     </row>
@@ -1070,28 +1070,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bungkam PSMS Medan 4-1, Persija Jakarta buka kans ke semifinal Piala Presiden</t>
+          <t>Pergelaran kesenian balaganjur pada hari suci umat Hindu di Bali</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 19:04:32 +0700</t>
+          <t>Sat, 01 Aug 2026 20:11:17 +0700</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pesepak bola Persija Jakarta Denis Kolinger (kanan) berebut bola udara dengan pesepak bola PSMS Medan Angelo Meneses (kiri) dan Asyraq Gufron (tengah) pada pertandingan Grup B Piala Presiden 2026 di Stadion Gelora Bung Tomo, Surabaya, Jawa Timur.</t>
+          <t>Sejumlah pemuda menampilkan kesenian baleganjur pada Hari Suci Tumpek Krulut di The Blooms Bali, Tabanan, Bali.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5675900/bungkam-psms-medan-4-1-persija-jakarta-buka-kans-ke-semifinal-piala-presiden</t>
+          <t>https://www.antaranews.com/foto/5676007/pergelaran-kesenian-balaganjur-pada-hari-suci-umat-hindu-di-bali</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Bola-3.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Bali-2.jpg</t>
         </is>
       </c>
     </row>
@@ -1103,28 +1103,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pemasangan jaring apung penahan sampah di Sungai Lestari</t>
+          <t>Bungkam PSMS Medan 4-1, Persija Jakarta buka kans ke semifinal Piala Presiden</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 18:17:45 +0700</t>
+          <t>Sat, 01 Aug 2026 19:04:32 +0700</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Relawan sungai memasang jaring terapung penahan sampah atau trash boom di Sungai Jenes, Pajang, Laweyan, Solo, Jawa Tengah, Sabtu (1/8/2026). Pemkot Solo bekerja sama dengan United Nations Development Programme (UNDP) dan Clean Rivers meluncurkan program penanganan sampah Sungai Lestari dengan skema sampah yang diambil dari hulu sungai Kota Solo akan langsung dipilah dan diolah oleh mitra lokal hingga diharapkan mampu menciptakan sungai yang yang bersih sekaligus upaya mengurangi beban kuota sampah di TPA Putri Cempo. ANTARA FOTO/Mohammad Ayudha/YU</t>
+          <t>Pesepak bola Persija Jakarta Denis Kolinger (kanan) berebut bola udara dengan pesepak bola PSMS Medan Angelo Meneses (kiri) dan Asyraq Gufron (tengah) pada pertandingan Grup B Piala Presiden 2026 di Stadion Gelora Bung Tomo, Surabaya, Jawa Timur.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5675871/pemasangan-jaring-apung-penahan-sampah-di-sungai-lestari</t>
+          <t>https://www.antaranews.com/foto/5675900/bungkam-psms-medan-4-1-persija-jakarta-buka-kans-ke-semifinal-piala-presiden</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/pemasangan-trash-boom-penahan-sampah-010826-yud-3.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Bola-3.jpg</t>
         </is>
       </c>
     </row>
@@ -1136,28 +1136,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Begini kemeriahan Jakarta Watersport Festival 2026 di Danau Sunter</t>
+          <t>Pemasangan jaring apung penahan sampah di Sungai Lestari</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sat, 01 Aug 2026 18:01:11 +0700</t>
+          <t>Sat, 01 Aug 2026 18:17:45 +0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Peserta beradu kecepatan saat mengikuti lomba perahu naga pada Jakarta Watersport Festival 2026 di Danau Sunter, Jakarta.</t>
+          <t>Relawan sungai memasang jaring terapung penahan sampah atau trash boom di Sungai Jenes, Pajang, Laweyan, Solo, Jawa Tengah, Sabtu (1/8/2026). Pemkot Solo bekerja sama dengan United Nations Development Programme (UNDP) dan Clean Rivers meluncurkan program penanganan sampah Sungai Lestari dengan skema sampah yang diambil dari hulu sungai Kota Solo akan langsung dipilah dan diolah oleh mitra lokal hingga diharapkan mampu menciptakan sungai yang yang bersih sekaligus upaya mengurangi beban kuota sampah di TPA Putri Cempo. ANTARA FOTO/Mohammad Ayudha/YU</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5675857/begini-kemeriahan-jakarta-watersport-festival-2026-di-danau-sunter</t>
+          <t>https://www.antaranews.com/foto/5675871/pemasangan-jaring-apung-penahan-sampah-di-sungai-lestari</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/Jakarta-Watersport-Festival-2026-182026-pma-2.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/01/pemasangan-trash-boom-penahan-sampah-010826-yud-3.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>